<commit_message>
Add OSB exposure analysis
</commit_message>
<xml_diff>
--- a/reports/model_comparison.xlsx
+++ b/reports/model_comparison.xlsx
@@ -420,16 +420,16 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.4808551654807863</v>
+        <v>0.5247158344991233</v>
       </c>
       <c r="C2">
-        <v>0.03798174035999548</v>
+        <v>0.0190740966818743</v>
       </c>
       <c r="D2">
-        <v>0.4728706692387029</v>
+        <v>0.4667734553775744</v>
       </c>
       <c r="E2">
-        <v>0.839622641509434</v>
+        <v>0.8773584905660378</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -437,16 +437,16 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.4643650402040179</v>
+        <v>0.4967124235200484</v>
       </c>
       <c r="C3">
-        <v>0.03753982867376204</v>
+        <v>0.03024872671020067</v>
       </c>
       <c r="D3">
-        <v>0.4315009010182592</v>
+        <v>0.4726450774959699</v>
       </c>
       <c r="E3">
-        <v>0.8930817610062893</v>
+        <v>0.8946540880503144</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -454,16 +454,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>0.4453723366432126</v>
+        <v>0.4374680184169586</v>
       </c>
       <c r="C4">
-        <v>0.04158231901885009</v>
+        <v>0.04795899476033678</v>
       </c>
       <c r="D4">
-        <v>0.4281211832049213</v>
+        <v>0.3957874762472464</v>
       </c>
       <c r="E4">
-        <v>0.8128930817610063</v>
+        <v>0.7704402515723271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrate 2024 data and executed notebooks
</commit_message>
<xml_diff>
--- a/reports/model_comparison.xlsx
+++ b/reports/model_comparison.xlsx
@@ -420,16 +420,16 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.5247158344991233</v>
+        <v>0.5057073391834982</v>
       </c>
       <c r="C2">
-        <v>0.0190740966818743</v>
+        <v>0.01386485272459466</v>
       </c>
       <c r="D2">
-        <v>0.4667734553775744</v>
+        <v>0.5087669934038649</v>
       </c>
       <c r="E2">
-        <v>0.8773584905660378</v>
+        <v>0.8979591836734694</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -437,16 +437,16 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.4967124235200484</v>
+        <v>0.4691452875366163</v>
       </c>
       <c r="C3">
-        <v>0.03024872671020067</v>
+        <v>0.04113219543897138</v>
       </c>
       <c r="D3">
-        <v>0.4726450774959699</v>
+        <v>0.465310278355645</v>
       </c>
       <c r="E3">
-        <v>0.8946540880503144</v>
+        <v>0.9056122448979592</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -454,16 +454,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>0.4374680184169586</v>
+        <v>0.419464808063081</v>
       </c>
       <c r="C4">
-        <v>0.04795899476033678</v>
+        <v>0.01305677819705672</v>
       </c>
       <c r="D4">
-        <v>0.3957874762472464</v>
+        <v>0.4309854757714449</v>
       </c>
       <c r="E4">
-        <v>0.7704402515723271</v>
+        <v>0.7933673469387755</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add national weather enrichment
</commit_message>
<xml_diff>
--- a/reports/model_comparison.xlsx
+++ b/reports/model_comparison.xlsx
@@ -420,16 +420,16 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.5057073391834982</v>
+        <v>0.4955005340579427</v>
       </c>
       <c r="C2">
-        <v>0.01386485272459466</v>
+        <v>0.02246577547610419</v>
       </c>
       <c r="D2">
-        <v>0.5087669934038649</v>
+        <v>0.5277547557777935</v>
       </c>
       <c r="E2">
-        <v>0.8979591836734694</v>
+        <v>0.9053177691309987</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -437,16 +437,16 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.4691452875366163</v>
+        <v>0.4421579785056016</v>
       </c>
       <c r="C3">
-        <v>0.04113219543897138</v>
+        <v>0.03095073112843591</v>
       </c>
       <c r="D3">
-        <v>0.465310278355645</v>
+        <v>0.4780004118086119</v>
       </c>
       <c r="E3">
-        <v>0.9056122448979592</v>
+        <v>0.9130998702983139</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -454,16 +454,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>0.419464808063081</v>
+        <v>0.4197168156116697</v>
       </c>
       <c r="C4">
-        <v>0.01305677819705672</v>
+        <v>0.01483311107853384</v>
       </c>
       <c r="D4">
-        <v>0.4309854757714449</v>
+        <v>0.4255008491092186</v>
       </c>
       <c r="E4">
-        <v>0.7933673469387755</v>
+        <v>0.7833981841763943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>